<commit_message>
Read every format through the new readers by its dialect
</commit_message>
<xml_diff>
--- a/tests/data/synthetic-layouts/layouts.xlsx
+++ b/tests/data/synthetic-layouts/layouts.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H3" s="2" t="n"/>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>

</xml_diff>